<commit_message>
Updated IND_grids_kan model - 2026-05-13 18:18
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan/SuppXLS/Scen_advanced_features.xlsx
+++ b/VerveStacks_IND_grids_kan/SuppXLS/Scen_advanced_features.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824B08BC-82CE-42B4-80F3-1F3B80C4BED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88199344-6D9C-45B5-B9E0-E8F0DE186FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
+    <workbookView xWindow="28702" yWindow="-98" windowWidth="28995" windowHeight="15675" activeTab="4" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
   </bookViews>
   <sheets>
     <sheet name="veda input" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="248">
   <si>
     <t>ACT_MINLD</t>
   </si>
@@ -2596,21 +2596,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> can be challenging if oil seeped into ground over years. Oil can create a long-term pollution plume, so regulations require thorough cleanup (soil excavation or in-situ treatment) in many jurisdictions. This is labor- and cost-intensive and is often the largest single cost item, much like coal ash is for coal plants. Salvage helps (old oil tanks can be scrapped, equipment sold), but it may not offset the high cleanup costs. Uncertainty is high, hinging on how contaminated the site is. Some old oil plants that operated only sparingly may have minimal contamination and thus be relatively cheap to retire (~$30–40/kW), whereas others that ran for decades and leaked oil could be at the upper end or beyond.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Sources:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All cost estimates are derived from industry reports and case studies. For example, Raimi (2017) provides average and range for U.S. plant decommissioning costs by fuel, which we have updated to 2023 USD. Additional data from World Bank/ESMAP, Gold Standard, NewClimate Institute, and World Nuclear Association/IAEA inform the figures. Where specific technologies have not yet been decommissioned (e.g. CCS-equipped plants, SMRs), we have indicated that no direct sources exist and provided reasoned estimates (with assumptions noted). All ranges reflect low/high scenarios; higher-end costs usually assume more extensive environmental remediation per regional regulatory requirements.</t>
     </r>
   </si>
   <si>
@@ -2948,6 +2933,81 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>545307</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>176211</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2976562</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>4763</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0BDC4EF9-5E8A-2F58-6455-1CFB661B4753}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="545307" y="40285986"/>
+          <a:ext cx="8170068" cy="1276352"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-IN" sz="1100"/>
+            <a:t>Sources: All cost estimates are derived from industry reports and case studies. For example, Raimi (2017) provides average and range for U.S. plant decommissioning costs by fuel, which we have updated to 2023 USD. Additional data from World Bank/ESMAP, Gold Standard, NewClimate Institute, and World Nuclear Association/IAEA inform the figures. Where specific technologies have not yet been decommissioned (e.g. CCS-equipped plants, SMRs), we have indicated that no direct sources exist and provided reasoned estimates (with assumptions noted). All ranges reflect low/high scenarios; higher-end costs usually assume more extensive environmental remediation per regional regulatory requirements.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3273,7 +3333,7 @@
   <sheetData>
     <row r="2" spans="2:19" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="D2" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="N2" s="2" t="s">
         <v>90</v>
@@ -3311,7 +3371,7 @@
         <v>82</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="M3" s="9"/>
       <c r="N3" s="3" t="s">
@@ -4073,7 +4133,7 @@
         <v>0.1</v>
       </c>
       <c r="H17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>83</v>
@@ -4162,39 +4222,39 @@
   <sheetData>
     <row r="2" spans="2:50" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="AD2" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="3" spans="2:50" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" t="s">
         <v>203</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>204</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>205</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>206</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>207</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>208</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>209</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>210</v>
-      </c>
-      <c r="J3" t="s">
-        <v>211</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -4242,7 +4302,7 @@
         <v>200</v>
       </c>
       <c r="AD3" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AE3" s="3">
         <f t="shared" ref="AE3:AS4" si="0">K3</f>
@@ -4307,25 +4367,25 @@
     </row>
     <row r="4" spans="2:50" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C4" t="s">
         <v>213</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>214</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>214</v>
+      </c>
+      <c r="F4" t="s">
         <v>215</v>
-      </c>
-      <c r="E4" t="s">
-        <v>215</v>
-      </c>
-      <c r="F4" t="s">
-        <v>216</v>
       </c>
       <c r="G4" s="17">
         <v>39.18</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I4" s="17">
         <v>43.5</v>
@@ -4445,25 +4505,25 @@
     </row>
     <row r="5" spans="2:50" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
+        <v>217</v>
+      </c>
+      <c r="C5" t="s">
+        <v>214</v>
+      </c>
+      <c r="D5" t="s">
         <v>218</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F5" t="s">
         <v>215</v>
-      </c>
-      <c r="D5" t="s">
-        <v>219</v>
-      </c>
-      <c r="E5" t="s">
-        <v>215</v>
-      </c>
-      <c r="F5" t="s">
-        <v>216</v>
       </c>
       <c r="G5" s="17">
         <v>19.34</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="I5" s="17">
         <v>28.67</v>
@@ -4583,30 +4643,30 @@
     </row>
     <row r="7" spans="2:50" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="AD7" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" spans="2:50" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" t="s">
         <v>203</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>204</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>205</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>206</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>207</v>
       </c>
-      <c r="G8" t="s">
-        <v>208</v>
-      </c>
       <c r="H8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -4669,7 +4729,7 @@
         <v>200</v>
       </c>
       <c r="AD8" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AE8" s="3">
         <f t="shared" ref="AE8:AT10" si="2">I8</f>
@@ -4754,19 +4814,19 @@
     </row>
     <row r="9" spans="2:50" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
+        <v>219</v>
+      </c>
+      <c r="C9" t="s">
+        <v>214</v>
+      </c>
+      <c r="D9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E9" t="s">
+        <v>214</v>
+      </c>
+      <c r="F9" t="s">
         <v>220</v>
-      </c>
-      <c r="C9" t="s">
-        <v>215</v>
-      </c>
-      <c r="D9" t="s">
-        <v>215</v>
-      </c>
-      <c r="E9" t="s">
-        <v>215</v>
-      </c>
-      <c r="F9" t="s">
-        <v>221</v>
       </c>
       <c r="G9" s="17">
         <v>30.18</v>
@@ -4921,19 +4981,19 @@
     </row>
     <row r="10" spans="2:50" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G10" s="17">
         <v>19.73</v>
@@ -5088,47 +5148,47 @@
     </row>
     <row r="13" spans="2:50" x14ac:dyDescent="0.45">
       <c r="B13" s="16" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" spans="2:50" x14ac:dyDescent="0.45">
       <c r="B14" s="18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C14" s="18"/>
       <c r="D14" s="18"/>
     </row>
     <row r="15" spans="2:50" x14ac:dyDescent="0.45">
       <c r="B15" s="18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="18"/>
     </row>
     <row r="16" spans="2:50" x14ac:dyDescent="0.45">
       <c r="B16" s="18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="18"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B18" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="C18" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="D18" s="18" t="s">
         <v>228</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B19" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="C19" s="18" t="s">
         <v>230</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>231</v>
       </c>
       <c r="D19" s="18">
         <v>253</v>
@@ -5136,36 +5196,36 @@
     </row>
     <row r="20" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B20" s="18" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D20" s="18">
         <v>203</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="21" spans="2:12" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B21" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>234</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>235</v>
       </c>
       <c r="D21" s="18">
         <v>82</v>
       </c>
       <c r="H21" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I21" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="J21" s="3" t="s">
         <v>237</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>238</v>
       </c>
       <c r="K21" s="3">
         <v>2019</v>
@@ -5176,22 +5236,22 @@
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B22" s="18" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D22" s="18">
         <v>242</v>
       </c>
       <c r="H22" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I22" t="s">
+        <v>245</v>
+      </c>
+      <c r="J22" t="s">
         <v>246</v>
-      </c>
-      <c r="J22" t="s">
-        <v>247</v>
       </c>
       <c r="K22">
         <f>AD4</f>
@@ -5203,16 +5263,16 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B23" s="18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D23" s="18">
         <v>226</v>
       </c>
       <c r="H23" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I23" t="s">
         <v>80</v>
@@ -5227,16 +5287,16 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B24" s="18" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D24" s="18">
         <v>174</v>
       </c>
       <c r="H24" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I24" t="s">
         <v>22</v>
@@ -5251,16 +5311,16 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B25" s="18" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D25" s="18">
         <v>258</v>
       </c>
       <c r="H25" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I25" t="s">
         <v>15</v>
@@ -5275,10 +5335,10 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B26" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="C26" s="18" t="s">
         <v>244</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>245</v>
       </c>
       <c r="D26" s="18">
         <v>135</v>
@@ -5967,7 +6027,7 @@
         <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
@@ -6501,12 +6561,11 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A25" s="15" t="s">
-        <v>197</v>
-      </c>
+      <c r="A25" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>